<commit_message>
Daily NSE scan: 2026-09-29
</commit_message>
<xml_diff>
--- a/output/2026-09-29/enriched_analysis.xlsx
+++ b/output/2026-09-29/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>3.374</v>
+        <v>3.349</v>
       </c>
       <c r="W2" t="n">
-        <v>2846</v>
+        <v>2867</v>
       </c>
       <c r="X2" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.873</v>
+        <v>0.902</v>
       </c>
       <c r="W3" t="n">
-        <v>346</v>
+        <v>335</v>
       </c>
       <c r="X3" t="n">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="Y3" t="n">
         <v>22</v>
@@ -1393,10 +1393,10 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.962</v>
       </c>
       <c r="W4" t="n">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="n">
@@ -1626,10 +1626,10 @@
         <v>0.052</v>
       </c>
       <c r="W5" t="n">
-        <v>2565</v>
+        <v>2543</v>
       </c>
       <c r="X5" t="n">
-        <v>8.82</v>
+        <v>8.74</v>
       </c>
       <c r="Y5" t="n">
         <v>36</v>
@@ -1855,13 +1855,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0.119</v>
+        <v>0.12</v>
       </c>
       <c r="W6" t="n">
-        <v>2632</v>
+        <v>2627</v>
       </c>
       <c r="X6" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="Y6" t="n">
         <v>-3</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.444</v>
+        <v>0.448</v>
       </c>
       <c r="W7" t="n">
-        <v>2745</v>
+        <v>2719</v>
       </c>
       <c r="X7" t="n">
-        <v>22.5</v>
+        <v>22.3</v>
       </c>
       <c r="Y7" t="n">
         <v>8</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.988</v>
+        <v>0.96</v>
       </c>
       <c r="W8" t="n">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="X8" t="n">
-        <v>8.640000000000001</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="Y8" t="n">
         <v>17</v>
@@ -2554,10 +2554,10 @@
         <v>0.05</v>
       </c>
       <c r="W9" t="n">
-        <v>1662</v>
+        <v>1654</v>
       </c>
       <c r="X9" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="Y9" t="n">
         <v>55</v>
@@ -2786,10 +2786,10 @@
         <v>0.313</v>
       </c>
       <c r="W10" t="n">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="X10" t="n">
-        <v>9.619999999999999</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="Y10" t="n">
         <v>7</v>
@@ -3245,13 +3245,13 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>0.046</v>
+        <v>0.047</v>
       </c>
       <c r="W12" t="n">
-        <v>15577</v>
+        <v>15367</v>
       </c>
       <c r="X12" t="n">
-        <v>39.7</v>
+        <v>39.1</v>
       </c>
       <c r="Y12" t="n">
         <v>83</v>
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>2.301</v>
+        <v>2.319</v>
       </c>
       <c r="W13" t="n">
-        <v>2551</v>
+        <v>2531</v>
       </c>
       <c r="X13" t="n">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="Y13" t="n">
         <v>6</v>
@@ -3709,13 +3709,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.13</v>
+        <v>0.118</v>
       </c>
       <c r="W14" t="n">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="X14" t="n">
-        <v>35.9</v>
+        <v>39.5</v>
       </c>
       <c r="Y14" t="n">
         <v>19</v>
@@ -3965,7 +3965,7 @@
         <v>1.58</v>
       </c>
       <c r="AD15" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE15" t="b">
         <v>0</v>
@@ -4101,16 +4101,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -4118,40 +4118,40 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G16" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H16" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>189.43</v>
+        <v>387.2</v>
       </c>
       <c r="J16" t="n">
-        <v>170.45</v>
+        <v>338.1</v>
       </c>
       <c r="K16" t="n">
-        <v>11.1</v>
+        <v>14.5</v>
       </c>
       <c r="L16" t="n">
-        <v>67.54000000000001</v>
+        <v>66.73</v>
       </c>
       <c r="M16" t="n">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="N16" t="n">
-        <v>2560187</v>
+        <v>3381000</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>2560187</v>
+        <v>3381000</v>
       </c>
       <c r="Q16" t="n">
         <v>0</v>
@@ -4165,69 +4165,69 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.1</v>
+        <v>0.074</v>
       </c>
       <c r="W16" t="n">
-        <v>255</v>
+        <v>456</v>
       </c>
       <c r="X16" t="n">
-        <v>27.3</v>
+        <v>13.5</v>
       </c>
       <c r="Y16" t="n">
+        <v>-8</v>
+      </c>
+      <c r="Z16" t="n">
         <v>24</v>
       </c>
-      <c r="Z16" t="n">
-        <v>1.87</v>
-      </c>
       <c r="AA16" t="n">
-        <v>-31</v>
+        <v>33</v>
       </c>
       <c r="AB16" t="n">
-        <v>3.36</v>
+        <v>14.36</v>
       </c>
       <c r="AC16" t="n">
-        <v>4.96</v>
+        <v>9.94</v>
       </c>
       <c r="AD16" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="AE16" t="b">
         <v>1</v>
       </c>
       <c r="AF16" t="n">
-        <v>2.97</v>
+        <v>18</v>
       </c>
       <c r="AG16" t="n">
-        <v>181.38</v>
+        <v>362.06</v>
       </c>
       <c r="AH16" t="n">
-        <v>163.89</v>
+        <v>270.72</v>
       </c>
       <c r="AI16" t="n">
-        <v>56.1</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="AJ16" t="n">
-        <v>170.4518641810919</v>
+        <v>338.1</v>
       </c>
       <c r="AK16" t="n">
-        <v>11.1</v>
+        <v>14.5</v>
       </c>
       <c r="AL16" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM16" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN16" t="inlineStr">
@@ -4237,22 +4237,22 @@
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AQ16" t="n">
         <v>0</v>
       </c>
       <c r="AR16" t="n">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="AS16" t="n">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="AT16" t="n">
         <v>0</v>
@@ -4261,13 +4261,13 @@
         <v>0</v>
       </c>
       <c r="AV16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AW16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY16" t="n">
         <v>0</v>
@@ -4276,13 +4276,13 @@
         <v>0</v>
       </c>
       <c r="BA16" t="n">
-        <v>2560187</v>
+        <v>0</v>
       </c>
       <c r="BB16" t="n">
-        <v>2560187</v>
+        <v>3381000</v>
       </c>
       <c r="BC16" t="n">
-        <v>2560187</v>
+        <v>3381000</v>
       </c>
       <c r="BD16" t="n">
         <v>0</v>
@@ -4318,10 +4318,10 @@
         <v>0</v>
       </c>
       <c r="BO16" t="n">
-        <v>2560187</v>
+        <v>0</v>
       </c>
       <c r="BP16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ16" t="n">
         <v>0</v>
@@ -4333,12 +4333,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>Savita Oil Technologies Limited</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -4350,279 +4350,279 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="G17" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="I17" t="n">
-        <v>387.2</v>
+        <v>699.3</v>
       </c>
       <c r="J17" t="n">
-        <v>338.1</v>
+        <v>726.25</v>
       </c>
       <c r="K17" t="n">
-        <v>14.5</v>
+        <v>-3.7</v>
       </c>
       <c r="L17" t="n">
-        <v>66.73</v>
+        <v>71.92</v>
       </c>
       <c r="M17" t="n">
-        <v>0.34</v>
+        <v>3.76</v>
       </c>
       <c r="N17" t="n">
-        <v>3381000</v>
+        <v>37641643</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>37427640</v>
       </c>
       <c r="P17" t="n">
-        <v>3381000</v>
+        <v>214003</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>99.43000000000001</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Net Buying</t>
+          <t>Net Buying with Selling</t>
         </is>
       </c>
       <c r="S17" t="b">
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.074</v>
+        <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>456</v>
+        <v>4826</v>
       </c>
       <c r="X17" t="n">
-        <v>13.5</v>
+        <v>11.3</v>
       </c>
       <c r="Y17" t="n">
-        <v>-8</v>
+        <v>26</v>
       </c>
       <c r="Z17" t="n">
-        <v>24</v>
+        <v>364</v>
       </c>
       <c r="AA17" t="n">
-        <v>33</v>
+        <v>204</v>
       </c>
       <c r="AB17" t="n">
-        <v>14.36</v>
+        <v>42.63</v>
       </c>
       <c r="AC17" t="n">
-        <v>9.94</v>
+        <v>14</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="AE17" t="b">
         <v>1</v>
       </c>
       <c r="AF17" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="AG17" t="n">
-        <v>362.06</v>
+        <v>685.42</v>
       </c>
       <c r="AH17" t="n">
-        <v>270.72</v>
+        <v>478.79</v>
       </c>
       <c r="AI17" t="n">
-        <v>95.40000000000001</v>
+        <v>112.4</v>
       </c>
       <c r="AJ17" t="n">
-        <v>338.1</v>
+        <v>726.2520355006753</v>
       </c>
       <c r="AK17" t="n">
-        <v>14.5</v>
+        <v>-3.7</v>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AQ17" t="n">
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="AS17" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="AT17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>37641643</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>37641643</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>37641643</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>37641643</v>
+      </c>
+      <c r="BC17" t="n">
+        <v>37641643</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>37427640</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>37427640</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>37427640</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>37427640</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>37427640</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>214003</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>214003</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR17" t="n">
         <v>1</v>
-      </c>
-      <c r="AX17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB17" t="n">
-        <v>3381000</v>
-      </c>
-      <c r="BC17" t="n">
-        <v>3381000</v>
-      </c>
-      <c r="BD17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR17" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Savita Oil Technologies Limited</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>Fundamental Watch</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="G18" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H18" t="n">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="I18" t="n">
-        <v>699.3</v>
+        <v>189.43</v>
       </c>
       <c r="J18" t="n">
-        <v>726.25</v>
+        <v>170.45</v>
       </c>
       <c r="K18" t="n">
-        <v>-3.7</v>
+        <v>11.1</v>
       </c>
       <c r="L18" t="n">
-        <v>71.92</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="M18" t="n">
-        <v>3.76</v>
+        <v>0.26</v>
       </c>
       <c r="N18" t="n">
-        <v>37641643</v>
+        <v>2560187</v>
       </c>
       <c r="O18" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>214003</v>
+        <v>2560187</v>
       </c>
       <c r="Q18" t="n">
-        <v>99.43000000000001</v>
+        <v>0</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Net Buying with Selling</t>
+          <t>Net Buying</t>
         </is>
       </c>
       <c r="S18" t="b">
@@ -4633,32 +4633,32 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0</v>
+        <v>0.098</v>
       </c>
       <c r="W18" t="n">
-        <v>4794</v>
+        <v>260</v>
       </c>
       <c r="X18" t="n">
-        <v>11.2</v>
+        <v>27.8</v>
       </c>
       <c r="Y18" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="Z18" t="n">
-        <v>364</v>
+        <v>1.87</v>
       </c>
       <c r="AA18" t="n">
-        <v>204</v>
+        <v>-31</v>
       </c>
       <c r="AB18" t="n">
-        <v>42.63</v>
+        <v>3.36</v>
       </c>
       <c r="AC18" t="n">
-        <v>14</v>
+        <v>4.96</v>
       </c>
       <c r="AD18" t="n">
         <v>0</v>
@@ -4667,62 +4667,62 @@
         <v>1</v>
       </c>
       <c r="AF18" t="n">
-        <v>25</v>
+        <v>2.97</v>
       </c>
       <c r="AG18" t="n">
-        <v>685.42</v>
+        <v>181.38</v>
       </c>
       <c r="AH18" t="n">
-        <v>478.79</v>
+        <v>163.89</v>
       </c>
       <c r="AI18" t="n">
-        <v>112.4</v>
+        <v>56.1</v>
       </c>
       <c r="AJ18" t="n">
-        <v>726.2520355006753</v>
+        <v>170.4518641810919</v>
       </c>
       <c r="AK18" t="n">
-        <v>-3.7</v>
+        <v>11.1</v>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AQ18" t="n">
         <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="AS18" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="AT18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV18" t="n">
         <v>2</v>
@@ -4734,64 +4734,64 @@
         <v>2</v>
       </c>
       <c r="AY18" t="n">
-        <v>37641643</v>
+        <v>0</v>
       </c>
       <c r="AZ18" t="n">
-        <v>37641643</v>
+        <v>0</v>
       </c>
       <c r="BA18" t="n">
-        <v>37641643</v>
+        <v>2560187</v>
       </c>
       <c r="BB18" t="n">
-        <v>37641643</v>
+        <v>2560187</v>
       </c>
       <c r="BC18" t="n">
-        <v>37641643</v>
+        <v>2560187</v>
       </c>
       <c r="BD18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BE18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BF18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BH18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BI18" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BJ18" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BK18" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BL18" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BM18" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BN18" t="n">
-        <v>214003</v>
+        <v>0</v>
       </c>
       <c r="BO18" t="n">
-        <v>214003</v>
+        <v>2560187</v>
       </c>
       <c r="BP18" t="n">
         <v>2</v>
       </c>
       <c r="BQ18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BR18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -4869,13 +4869,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.132</v>
+        <v>0.133</v>
       </c>
       <c r="W19" t="n">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="X19" t="n">
-        <v>6.08</v>
+        <v>6.02</v>
       </c>
       <c r="Y19" t="n">
         <v>118</v>
@@ -5097,13 +5097,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>2.869</v>
+        <v>2.885</v>
       </c>
       <c r="W20" t="n">
-        <v>686</v>
+        <v>682</v>
       </c>
       <c r="X20" t="n">
-        <v>25.8</v>
+        <v>25.6</v>
       </c>
       <c r="Y20" t="n">
         <v>30</v>
@@ -5558,10 +5558,10 @@
         <v>0.083</v>
       </c>
       <c r="W22" t="n">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="X22" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="Y22" t="n">
         <v>-5</v>
@@ -5790,7 +5790,7 @@
         <v>0.024</v>
       </c>
       <c r="W23" t="n">
-        <v>1011</v>
+        <v>1034</v>
       </c>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="n">
@@ -6017,13 +6017,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.059</v>
+        <v>0.06</v>
       </c>
       <c r="W24" t="n">
-        <v>1849</v>
+        <v>1827</v>
       </c>
       <c r="X24" t="n">
-        <v>42.4</v>
+        <v>41.9</v>
       </c>
       <c r="Y24" t="n">
         <v>20</v>
@@ -6249,13 +6249,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.051</v>
+        <v>0.052</v>
       </c>
       <c r="W25" t="n">
-        <v>5144</v>
+        <v>5084</v>
       </c>
       <c r="X25" t="n">
-        <v>33.5</v>
+        <v>33.1</v>
       </c>
       <c r="Y25" t="n">
         <v>-25</v>
@@ -6481,13 +6481,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.897</v>
+        <v>0.918</v>
       </c>
       <c r="W26" t="n">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="X26" t="n">
-        <v>6.48</v>
+        <v>6.31</v>
       </c>
       <c r="Y26" t="n">
         <v>31</v>
@@ -6712,7 +6712,7 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="W27" t="n">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="X27" t="n">
         <v>20</v>
@@ -6939,13 +6939,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.17</v>
+        <v>0.167</v>
       </c>
       <c r="W28" t="n">
-        <v>652</v>
+        <v>664</v>
       </c>
       <c r="X28" t="n">
-        <v>54.5</v>
+        <v>55.5</v>
       </c>
       <c r="Y28" t="n">
         <v>3</v>
@@ -7171,13 +7171,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.65</v>
+        <v>0.647</v>
       </c>
       <c r="W29" t="n">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="X29" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="Y29" t="n">
         <v>19</v>
@@ -7403,13 +7403,13 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>0.497</v>
+        <v>0.491</v>
       </c>
       <c r="W30" t="n">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="X30" t="n">
-        <v>37.5</v>
+        <v>37.9</v>
       </c>
       <c r="Y30" t="n">
         <v>-44</v>
@@ -7635,13 +7635,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.658</v>
+        <v>0.654</v>
       </c>
       <c r="W31" t="n">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="X31" t="n">
-        <v>1152</v>
+        <v>1157</v>
       </c>
       <c r="Y31" t="n">
         <v>-61</v>
@@ -8098,10 +8098,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W33" t="n">
-        <v>52802</v>
+        <v>52721</v>
       </c>
       <c r="X33" t="n">
-        <v>44.7</v>
+        <v>44.6</v>
       </c>
       <c r="Y33" t="n">
         <v>5</v>
@@ -8327,13 +8327,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.02</v>
+        <v>0.021</v>
       </c>
       <c r="W34" t="n">
-        <v>9572</v>
+        <v>9489</v>
       </c>
       <c r="X34" t="n">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="Y34" t="n">
         <v>-12</v>
@@ -8559,13 +8559,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.804</v>
+        <v>0.805</v>
       </c>
       <c r="W35" t="n">
-        <v>3929</v>
+        <v>3923</v>
       </c>
       <c r="X35" t="n">
-        <v>27.5</v>
+        <v>27.4</v>
       </c>
       <c r="Y35" t="n">
         <v>2</v>
@@ -8794,10 +8794,10 @@
         <v>0.008</v>
       </c>
       <c r="W36" t="n">
-        <v>5217</v>
+        <v>5401</v>
       </c>
       <c r="X36" t="n">
-        <v>8.82</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="Y36" t="n">
         <v>43</v>
@@ -9026,10 +9026,10 @@
         <v>0.04</v>
       </c>
       <c r="W37" t="n">
-        <v>3388</v>
+        <v>3363</v>
       </c>
       <c r="X37" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="Y37" t="n">
         <v>-4</v>
@@ -9255,13 +9255,13 @@
         </is>
       </c>
       <c r="V38" t="n">
-        <v>0.221</v>
+        <v>0.224</v>
       </c>
       <c r="W38" t="n">
-        <v>632</v>
+        <v>624</v>
       </c>
       <c r="X38" t="n">
-        <v>13.9</v>
+        <v>13.7</v>
       </c>
       <c r="Y38" t="n">
         <v>-1</v>
@@ -9716,10 +9716,10 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>3411</v>
+        <v>3357</v>
       </c>
       <c r="X40" t="n">
-        <v>76.8</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="Y40" t="n">
         <v>42</v>
@@ -9948,10 +9948,10 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>8823</v>
+        <v>8779</v>
       </c>
       <c r="X41" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="Y41" t="n">
         <v>21</v>
@@ -10407,13 +10407,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.216</v>
+        <v>0.218</v>
       </c>
       <c r="W43" t="n">
-        <v>946</v>
+        <v>939</v>
       </c>
       <c r="X43" t="n">
-        <v>25.8</v>
+        <v>25.6</v>
       </c>
       <c r="Y43" t="n">
         <v>9</v>
@@ -10639,13 +10639,13 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.213</v>
+        <v>0.221</v>
       </c>
       <c r="W44" t="n">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="X44" t="n">
-        <v>25.1</v>
+        <v>24.2</v>
       </c>
       <c r="Y44" t="n">
         <v>21</v>
@@ -10874,10 +10874,10 @@
         <v>0.044</v>
       </c>
       <c r="W45" t="n">
-        <v>1566</v>
+        <v>1563</v>
       </c>
       <c r="X45" t="n">
-        <v>20.5</v>
+        <v>20.4</v>
       </c>
       <c r="Y45" t="n">
         <v>10</v>
@@ -11103,13 +11103,13 @@
         </is>
       </c>
       <c r="V46" t="n">
-        <v>0.218</v>
+        <v>0.221</v>
       </c>
       <c r="W46" t="n">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="X46" t="n">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
       <c r="Y46" t="n">
         <v>16</v>
@@ -11335,13 +11335,13 @@
         </is>
       </c>
       <c r="V47" t="n">
-        <v>0.231</v>
+        <v>0.232</v>
       </c>
       <c r="W47" t="n">
-        <v>1730</v>
+        <v>1720</v>
       </c>
       <c r="X47" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="Y47" t="n">
         <v>-3</v>
@@ -11570,10 +11570,10 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>116249</v>
+        <v>115311</v>
       </c>
       <c r="X48" t="n">
-        <v>33.5</v>
+        <v>33.2</v>
       </c>
       <c r="Y48" t="n">
         <v>18</v>
@@ -11799,13 +11799,13 @@
         </is>
       </c>
       <c r="V49" t="n">
-        <v>0.358</v>
+        <v>0.346</v>
       </c>
       <c r="W49" t="n">
-        <v>391</v>
+        <v>405</v>
       </c>
       <c r="X49" t="n">
-        <v>96.7</v>
+        <v>100</v>
       </c>
       <c r="Y49" t="n">
         <v>246</v>
@@ -12034,10 +12034,10 @@
         <v>0.083</v>
       </c>
       <c r="W50" t="n">
-        <v>1658</v>
+        <v>1642</v>
       </c>
       <c r="X50" t="n">
-        <v>29.9</v>
+        <v>29.7</v>
       </c>
       <c r="Y50" t="n">
         <v>39</v>
@@ -12753,105 +12753,105 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>189.43</v>
+        <v>387.2</v>
       </c>
       <c r="D16" t="n">
-        <v>170.45</v>
+        <v>338.1</v>
       </c>
       <c r="E16" t="n">
-        <v>11.1</v>
+        <v>14.5</v>
       </c>
       <c r="F16" t="n">
-        <v>67.54000000000001</v>
+        <v>66.73</v>
       </c>
       <c r="G16" t="n">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>Savita Oil Technologies Limited</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>387.2</v>
+        <v>699.3</v>
       </c>
       <c r="D17" t="n">
-        <v>338.1</v>
+        <v>726.25</v>
       </c>
       <c r="E17" t="n">
-        <v>14.5</v>
+        <v>-3.7</v>
       </c>
       <c r="F17" t="n">
-        <v>66.73</v>
+        <v>71.92</v>
       </c>
       <c r="G17" t="n">
-        <v>0.34</v>
+        <v>3.76</v>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Savita Oil Technologies Limited</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>699.3</v>
+        <v>189.43</v>
       </c>
       <c r="D18" t="n">
-        <v>726.25</v>
+        <v>170.45</v>
       </c>
       <c r="E18" t="n">
-        <v>-3.7</v>
+        <v>11.1</v>
       </c>
       <c r="F18" t="n">
-        <v>71.92</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>3.76</v>
+        <v>0.26</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
@@ -14078,7 +14078,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -14098,7 +14098,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>